<commit_message>
Debug controller end-of-test conditions
</commit_message>
<xml_diff>
--- a/data processing/data/cycles/file tracking.xlsx
+++ b/data processing/data/cycles/file tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cfolinus/Documents/MIT/CMF FIDL/07 Control/soft-actuator-controller/data processing/data/cycles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D82788B-6C0A-8749-8466-82BF9CFAA844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F04537F5-1D5A-754D-80DE-B146C9CFFC09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="22260" windowHeight="20640" activeTab="1" xr2:uid="{701280C3-9FED-6B42-B428-FC9DB4595006}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="24900" windowHeight="20640" activeTab="1" xr2:uid="{701280C3-9FED-6B42-B428-FC9DB4595006}"/>
   </bookViews>
   <sheets>
     <sheet name="Trial results" sheetId="2" r:id="rId1"/>
@@ -3705,7 +3705,7 @@
         <v>10</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>224</v>
@@ -3728,7 +3728,7 @@
         <v>10</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>220</v>
@@ -3751,7 +3751,7 @@
         <v>10</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>218</v>
@@ -3774,7 +3774,7 @@
         <v>14</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>59</v>
@@ -3800,7 +3800,7 @@
         <v>14</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>212</v>
@@ -3829,7 +3829,7 @@
         <v>22</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>86</v>
@@ -3864,7 +3864,7 @@
         <v>22</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>89</v>
@@ -3881,7 +3881,7 @@
         <v>22</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>90</v>
@@ -3904,7 +3904,7 @@
         <v>22</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>87</v>
@@ -3924,7 +3924,7 @@
         <v>22</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>88</v>
@@ -3944,7 +3944,7 @@
         <v>26</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>201</v>
@@ -3964,7 +3964,7 @@
         <v>26</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>199</v>
@@ -3990,7 +3990,7 @@
         <v>26</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>197</v>
@@ -4016,7 +4016,7 @@
         <v>26</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>195</v>
@@ -4036,7 +4036,7 @@
         <v>26</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>193</v>
@@ -4059,7 +4059,7 @@
         <v>26</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>191</v>
@@ -4082,7 +4082,7 @@
         <v>26</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>189</v>
@@ -4105,7 +4105,7 @@
         <v>26</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>186</v>
@@ -4128,7 +4128,7 @@
         <v>26</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>184</v>
@@ -4151,7 +4151,7 @@
         <v>26</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>182</v>
@@ -4174,7 +4174,7 @@
         <v>30</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>180</v>
@@ -4200,7 +4200,7 @@
         <v>42</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>177</v>
@@ -4223,7 +4223,7 @@
         <v>42</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>174</v>
@@ -4243,7 +4243,7 @@
         <v>42</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>172</v>
@@ -4260,7 +4260,7 @@
         <v>33</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>170</v>
@@ -4283,7 +4283,7 @@
         <v>33</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>168</v>
@@ -4306,7 +4306,7 @@
         <v>33</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>165</v>

</xml_diff>

<commit_message>
Tune solenoid valves for 2x controllers
</commit_message>
<xml_diff>
--- a/data processing/data/cycles/file tracking.xlsx
+++ b/data processing/data/cycles/file tracking.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cfolinus/Documents/MIT/CMF FIDL/07 Control/soft-actuator-controller/data processing/data/cycles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F04537F5-1D5A-754D-80DE-B146C9CFFC09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A00C23F4-3022-954D-99A7-E71FC5B0129C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="24900" windowHeight="20640" activeTab="1" xr2:uid="{701280C3-9FED-6B42-B428-FC9DB4595006}"/>
   </bookViews>
@@ -1567,48 +1567,6 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="1" fontId="6" fillId="6" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1636,22 +1594,64 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="17" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="18" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="19" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="19" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="19" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2009,39 +2009,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="25">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="82" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="H1" s="70" t="s">
+      <c r="B1" s="83"/>
+      <c r="C1" s="83"/>
+      <c r="D1" s="83"/>
+      <c r="E1" s="83"/>
+      <c r="F1" s="83"/>
+      <c r="H1" s="84" t="s">
         <v>133</v>
       </c>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-      <c r="O1" s="70"/>
-      <c r="P1" s="70"/>
+      <c r="I1" s="84"/>
+      <c r="J1" s="84"/>
+      <c r="K1" s="84"/>
+      <c r="L1" s="84"/>
+      <c r="M1" s="84"/>
+      <c r="N1" s="84"/>
+      <c r="O1" s="84"/>
+      <c r="P1" s="84"/>
     </row>
     <row r="2" spans="1:17" s="41" customFormat="1" ht="17" customHeight="1" thickBot="1">
-      <c r="A2" s="80" t="s">
+      <c r="A2" s="94" t="s">
         <v>91</v>
       </c>
-      <c r="B2" s="81"/>
-      <c r="C2" s="81"/>
+      <c r="B2" s="95"/>
+      <c r="C2" s="95"/>
       <c r="D2" s="43" t="s">
         <v>92</v>
       </c>
-      <c r="E2" s="79" t="s">
+      <c r="E2" s="93" t="s">
         <v>93</v>
       </c>
-      <c r="F2" s="79"/>
+      <c r="F2" s="93"/>
       <c r="G2" s="40"/>
     </row>
     <row r="3" spans="1:17" s="42" customFormat="1" ht="60" customHeight="1">
@@ -2064,22 +2064,22 @@
         <v>137</v>
       </c>
       <c r="H3" s="41"/>
-      <c r="I3" s="71" t="s">
+      <c r="I3" s="85" t="s">
         <v>121</v>
       </c>
-      <c r="J3" s="72"/>
-      <c r="K3" s="73" t="s">
+      <c r="J3" s="86"/>
+      <c r="K3" s="87" t="s">
         <v>122</v>
       </c>
-      <c r="L3" s="74"/>
-      <c r="M3" s="75" t="s">
+      <c r="L3" s="88"/>
+      <c r="M3" s="89" t="s">
         <v>128</v>
       </c>
-      <c r="N3" s="76"/>
-      <c r="O3" s="77" t="s">
+      <c r="N3" s="90"/>
+      <c r="O3" s="91" t="s">
         <v>123</v>
       </c>
-      <c r="P3" s="78"/>
+      <c r="P3" s="92"/>
     </row>
     <row r="4" spans="1:17" ht="31" customHeight="1">
       <c r="A4" s="46" t="s">
@@ -2472,7 +2472,7 @@
         <v>614.4</v>
       </c>
       <c r="O12" s="17"/>
-      <c r="P12" s="82">
+      <c r="P12" s="68">
         <f>AVERAGE(P5:P10)</f>
         <v>609.79999999999995</v>
       </c>
@@ -3012,8 +3012,9 @@
     <col min="2" max="2" width="10.28515625" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.7109375" style="3" customWidth="1"/>
-    <col min="5" max="5" width="24.7109375" style="83" customWidth="1"/>
-    <col min="6" max="7" width="24.7109375" style="3" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" style="69" customWidth="1"/>
+    <col min="6" max="6" width="24.7109375" style="3" customWidth="1"/>
+    <col min="7" max="7" width="33.140625" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.140625" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="21.140625" style="3" customWidth="1"/>
     <col min="10" max="10" width="34.85546875" style="4" customWidth="1"/>
@@ -3024,78 +3025,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="17" customHeight="1">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="81" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="98"/>
-      <c r="C1" s="98"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="97"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="95" t="s">
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="80"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="96" t="s">
         <v>92</v>
       </c>
-      <c r="I1" s="95"/>
-      <c r="J1" s="95"/>
-      <c r="K1" s="94" t="s">
+      <c r="I1" s="96"/>
+      <c r="J1" s="96"/>
+      <c r="K1" s="98" t="s">
         <v>93</v>
       </c>
-      <c r="L1" s="94"/>
-      <c r="M1" s="93" t="s">
+      <c r="L1" s="98"/>
+      <c r="M1" s="97" t="s">
         <v>296</v>
       </c>
-      <c r="N1" s="93"/>
-      <c r="O1" s="93"/>
-      <c r="P1" s="93"/>
-    </row>
-    <row r="2" spans="1:21" s="87" customFormat="1" ht="35" customHeight="1">
-      <c r="A2" s="91" t="s">
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+    </row>
+    <row r="2" spans="1:21" s="73" customFormat="1" ht="35" customHeight="1">
+      <c r="A2" s="77" t="s">
         <v>295</v>
       </c>
-      <c r="B2" s="91" t="s">
+      <c r="B2" s="77" t="s">
         <v>94</v>
       </c>
-      <c r="C2" s="91" t="s">
+      <c r="C2" s="77" t="s">
         <v>95</v>
       </c>
-      <c r="D2" s="91" t="s">
+      <c r="D2" s="77" t="s">
         <v>294</v>
       </c>
-      <c r="E2" s="92" t="s">
+      <c r="E2" s="78" t="s">
         <v>293</v>
       </c>
-      <c r="F2" s="91" t="s">
+      <c r="F2" s="77" t="s">
         <v>292</v>
       </c>
-      <c r="G2" s="91" t="s">
+      <c r="G2" s="77" t="s">
         <v>291</v>
       </c>
-      <c r="H2" s="90" t="s">
+      <c r="H2" s="76" t="s">
         <v>290</v>
       </c>
-      <c r="I2" s="90" t="s">
+      <c r="I2" s="76" t="s">
         <v>289</v>
       </c>
-      <c r="J2" s="90" t="s">
+      <c r="J2" s="76" t="s">
         <v>137</v>
       </c>
-      <c r="K2" s="89" t="s">
+      <c r="K2" s="75" t="s">
         <v>288</v>
       </c>
-      <c r="L2" s="89" t="s">
+      <c r="L2" s="75" t="s">
         <v>287</v>
       </c>
-      <c r="M2" s="88" t="s">
+      <c r="M2" s="74" t="s">
         <v>286</v>
       </c>
-      <c r="N2" s="88" t="s">
+      <c r="N2" s="74" t="s">
         <v>285</v>
       </c>
-      <c r="O2" s="88" t="s">
+      <c r="O2" s="74" t="s">
         <v>284</v>
       </c>
-      <c r="P2" s="88" t="s">
+      <c r="P2" s="74" t="s">
         <v>283</v>
       </c>
       <c r="U2" s="3"/>
@@ -3113,7 +3114,7 @@
       <c r="D3" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E3" s="85" t="s">
+      <c r="E3" s="71" t="s">
         <v>32</v>
       </c>
       <c r="H3" s="4" t="s">
@@ -3151,7 +3152,7 @@
       <c r="D4" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="E4" s="83">
+      <c r="E4" s="69">
         <v>700</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -3192,7 +3193,7 @@
       <c r="D5" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="E5" s="83">
+      <c r="E5" s="69">
         <v>248</v>
       </c>
       <c r="F5" s="3" t="s">
@@ -3215,7 +3216,7 @@
       <c r="D6" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="E6" s="83">
+      <c r="E6" s="69">
         <v>176</v>
       </c>
       <c r="F6" s="3" t="s">
@@ -3238,7 +3239,7 @@
       <c r="D7" s="3" t="s">
         <v>273</v>
       </c>
-      <c r="E7" s="83">
+      <c r="E7" s="69">
         <v>46</v>
       </c>
       <c r="F7" s="3" t="s">
@@ -3261,7 +3262,7 @@
       <c r="D8" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="83">
+      <c r="E8" s="69">
         <v>520</v>
       </c>
       <c r="F8" s="3" t="s">
@@ -3291,7 +3292,7 @@
       <c r="D9" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="E9" s="83">
+      <c r="E9" s="69">
         <v>11</v>
       </c>
       <c r="F9" s="3" t="s">
@@ -3314,7 +3315,7 @@
       <c r="D10" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="E10" s="83">
+      <c r="E10" s="69">
         <v>98</v>
       </c>
       <c r="F10" s="3" t="s">
@@ -3337,7 +3338,7 @@
       <c r="D11" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="E11" s="83">
+      <c r="E11" s="69">
         <v>66</v>
       </c>
       <c r="F11" s="3" t="s">
@@ -3357,7 +3358,7 @@
       <c r="D12" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E12" s="83">
+      <c r="E12" s="69">
         <v>129</v>
       </c>
       <c r="F12" s="3" t="s">
@@ -3377,7 +3378,7 @@
       <c r="D13" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="E13" s="83">
+      <c r="E13" s="69">
         <v>118</v>
       </c>
       <c r="F13" s="3" t="s">
@@ -3394,10 +3395,10 @@
       <c r="C14" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D14" s="86" t="s">
+      <c r="D14" s="72" t="s">
         <v>259</v>
       </c>
-      <c r="E14" s="83">
+      <c r="E14" s="69">
         <v>16</v>
       </c>
       <c r="F14" s="3" t="s">
@@ -3423,10 +3424,10 @@
       <c r="C15" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D15" s="86" t="s">
+      <c r="D15" s="72" t="s">
         <v>254</v>
       </c>
-      <c r="E15" s="83">
+      <c r="E15" s="69">
         <v>475</v>
       </c>
       <c r="F15" s="3" t="s">
@@ -3452,7 +3453,7 @@
       <c r="D16" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E16" s="83">
+      <c r="E16" s="69">
         <v>877</v>
       </c>
       <c r="F16" s="3" t="s">
@@ -3475,7 +3476,7 @@
       <c r="D17" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="E17" s="83">
+      <c r="E17" s="69">
         <v>0</v>
       </c>
       <c r="H17" s="3" t="s">
@@ -3498,7 +3499,7 @@
       <c r="D18" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="E18" s="85" t="s">
+      <c r="E18" s="71" t="s">
         <v>32</v>
       </c>
       <c r="H18" s="4" t="s">
@@ -3533,7 +3534,7 @@
       <c r="D19" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E19" s="83">
+      <c r="E19" s="69">
         <v>574</v>
       </c>
       <c r="F19" s="3" t="s">
@@ -3577,7 +3578,7 @@
       <c r="D20" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E20" s="83">
+      <c r="E20" s="69">
         <v>229</v>
       </c>
       <c r="F20" s="3" t="s">
@@ -3615,7 +3616,7 @@
       <c r="D21" s="3" t="s">
         <v>237</v>
       </c>
-      <c r="E21" s="83">
+      <c r="E21" s="69">
         <v>303</v>
       </c>
       <c r="F21" s="3" t="s">
@@ -3641,7 +3642,7 @@
       <c r="D22" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="E22" s="83">
+      <c r="E22" s="69">
         <v>224</v>
       </c>
       <c r="F22" s="3" t="s">
@@ -3667,7 +3668,7 @@
       <c r="D23" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="E23" s="83">
+      <c r="E23" s="69">
         <v>351</v>
       </c>
       <c r="F23" s="3" t="s">
@@ -3690,7 +3691,7 @@
       <c r="D24" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="E24" s="83">
+      <c r="E24" s="69">
         <v>0</v>
       </c>
       <c r="H24" s="3" t="s">
@@ -3710,7 +3711,7 @@
       <c r="D25" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="E25" s="83" t="s">
+      <c r="E25" s="69" t="s">
         <v>206</v>
       </c>
       <c r="G25" s="3" t="s">
@@ -3733,7 +3734,7 @@
       <c r="D26" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="E26" s="83">
+      <c r="E26" s="69">
         <v>1671</v>
       </c>
       <c r="F26" s="3" t="s">
@@ -3756,7 +3757,7 @@
       <c r="D27" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="E27" s="83">
+      <c r="E27" s="69">
         <v>986</v>
       </c>
       <c r="F27" s="3" t="s">
@@ -3779,7 +3780,7 @@
       <c r="D28" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E28" s="83">
+      <c r="E28" s="69">
         <v>3000</v>
       </c>
       <c r="F28" s="3" t="s">
@@ -3805,7 +3806,7 @@
       <c r="D29" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="E29" s="83">
+      <c r="E29" s="69">
         <v>95</v>
       </c>
       <c r="F29" s="3" t="s">
@@ -3834,7 +3835,7 @@
       <c r="D30" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="E30" s="83">
+      <c r="E30" s="69">
         <v>716</v>
       </c>
       <c r="F30" s="3" t="s">
@@ -3869,7 +3870,7 @@
       <c r="D31" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="E31" s="83" t="s">
+      <c r="E31" s="69" t="s">
         <v>206</v>
       </c>
       <c r="H31" s="4" t="s">
@@ -3886,7 +3887,7 @@
       <c r="D32" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="E32" s="83">
+      <c r="E32" s="69">
         <v>2688</v>
       </c>
       <c r="F32" s="3" t="s">
@@ -3909,7 +3910,7 @@
       <c r="D33" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="E33" s="83">
+      <c r="E33" s="69">
         <v>245</v>
       </c>
       <c r="F33" s="3" t="s">
@@ -3929,7 +3930,7 @@
       <c r="D34" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E34" s="83">
+      <c r="E34" s="69">
         <v>917</v>
       </c>
       <c r="F34" s="3" t="s">
@@ -3949,7 +3950,7 @@
       <c r="D35" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="E35" s="83">
+      <c r="E35" s="69">
         <v>0</v>
       </c>
       <c r="H35" s="3" t="s">
@@ -3969,7 +3970,7 @@
       <c r="D36" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="E36" s="83">
+      <c r="E36" s="69">
         <v>2283</v>
       </c>
       <c r="F36" s="3" t="s">
@@ -3978,7 +3979,7 @@
       <c r="G36" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="H36" s="84" t="s">
+      <c r="H36" s="70" t="s">
         <v>198</v>
       </c>
       <c r="J36" s="4" t="s">
@@ -3995,7 +3996,7 @@
       <c r="D37" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="E37" s="83">
+      <c r="E37" s="69">
         <v>4380</v>
       </c>
       <c r="F37" s="3" t="s">
@@ -4004,7 +4005,7 @@
       <c r="G37" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="H37" s="84" t="s">
+      <c r="H37" s="70" t="s">
         <v>196</v>
       </c>
       <c r="J37" s="4" t="s">
@@ -4021,7 +4022,7 @@
       <c r="D38" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="E38" s="83">
+      <c r="E38" s="69">
         <v>1</v>
       </c>
       <c r="F38" s="3" t="s">
@@ -4041,7 +4042,7 @@
       <c r="D39" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="E39" s="83">
+      <c r="E39" s="69">
         <v>317</v>
       </c>
       <c r="F39" s="3" t="s">
@@ -4050,7 +4051,7 @@
       <c r="G39" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="H39" s="84" t="s">
+      <c r="H39" s="70" t="s">
         <v>192</v>
       </c>
     </row>
@@ -4064,7 +4065,7 @@
       <c r="D40" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="E40" s="83">
+      <c r="E40" s="69">
         <v>2035</v>
       </c>
       <c r="F40" s="3" t="s">
@@ -4087,7 +4088,7 @@
       <c r="D41" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="E41" s="83">
+      <c r="E41" s="69">
         <v>1124</v>
       </c>
       <c r="F41" s="3" t="s">
@@ -4096,7 +4097,7 @@
       <c r="G41" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="H41" s="84" t="s">
+      <c r="H41" s="70" t="s">
         <v>187</v>
       </c>
     </row>
@@ -4110,7 +4111,7 @@
       <c r="D42" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="E42" s="83">
+      <c r="E42" s="69">
         <v>1215</v>
       </c>
       <c r="F42" s="3" t="s">
@@ -4133,7 +4134,7 @@
       <c r="D43" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="E43" s="83">
+      <c r="E43" s="69">
         <v>877</v>
       </c>
       <c r="F43" s="3" t="s">
@@ -4142,7 +4143,7 @@
       <c r="G43" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="H43" s="84" t="s">
+      <c r="H43" s="70" t="s">
         <v>183</v>
       </c>
     </row>
@@ -4156,7 +4157,7 @@
       <c r="D44" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="E44" s="83">
+      <c r="E44" s="69">
         <v>255</v>
       </c>
       <c r="F44" s="3" t="s">
@@ -4179,7 +4180,7 @@
       <c r="D45" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="E45" s="83">
+      <c r="E45" s="69">
         <v>866</v>
       </c>
       <c r="F45" s="3" t="s">
@@ -4188,7 +4189,7 @@
       <c r="G45" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="H45" s="84" t="s">
+      <c r="H45" s="70" t="s">
         <v>179</v>
       </c>
       <c r="J45" s="4" t="s">
@@ -4205,7 +4206,7 @@
       <c r="D46" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="E46" s="83">
+      <c r="E46" s="69">
         <v>3808</v>
       </c>
       <c r="F46" s="3" t="s">
@@ -4228,7 +4229,7 @@
       <c r="D47" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="E47" s="83">
+      <c r="E47" s="69">
         <v>527</v>
       </c>
       <c r="F47" s="3" t="s">
@@ -4248,7 +4249,7 @@
       <c r="D48" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="E48" s="83">
+      <c r="E48" s="69">
         <v>0</v>
       </c>
       <c r="H48" s="3" t="s">
@@ -4265,7 +4266,7 @@
       <c r="D49" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="E49" s="83">
+      <c r="E49" s="69">
         <v>3068</v>
       </c>
       <c r="F49" s="3" t="s">
@@ -4288,7 +4289,7 @@
       <c r="D50" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="E50" s="83">
+      <c r="E50" s="69">
         <v>2550</v>
       </c>
       <c r="F50" s="3" t="s">
@@ -4311,7 +4312,7 @@
       <c r="D51" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="E51" s="83">
+      <c r="E51" s="69">
         <v>0</v>
       </c>
       <c r="H51" s="3" t="s">
@@ -4328,7 +4329,7 @@
       <c r="D52" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="E52" s="83">
+      <c r="E52" s="69">
         <v>1100</v>
       </c>
       <c r="F52" s="3" t="s">
@@ -4351,7 +4352,7 @@
       <c r="D53" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="E53" s="83">
+      <c r="E53" s="69">
         <v>37</v>
       </c>
       <c r="F53" s="3" t="s">
@@ -4374,7 +4375,7 @@
       <c r="D54" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="E54" s="83">
+      <c r="E54" s="69">
         <v>151</v>
       </c>
       <c r="F54" s="3" t="s">
@@ -4403,7 +4404,7 @@
       <c r="D55" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="E55" s="83">
+      <c r="E55" s="69">
         <v>570</v>
       </c>
       <c r="F55" s="3" t="s">
@@ -4429,7 +4430,7 @@
       <c r="D56" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E56" s="83">
+      <c r="E56" s="69">
         <v>22</v>
       </c>
       <c r="F56" s="3" t="s">
@@ -4455,7 +4456,7 @@
       <c r="D57" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E57" s="83">
+      <c r="E57" s="69">
         <v>674</v>
       </c>
       <c r="F57" s="3" t="s">
@@ -4496,7 +4497,7 @@
       <c r="D58" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="E58" s="83">
+      <c r="E58" s="69">
         <v>518</v>
       </c>
       <c r="F58" s="3" t="s">

</xml_diff>